<commit_message>
Deploy ResistAI QA Reports & Docs [build-20] - GitHub Pages bbdc56474953c34476e4ff956c4446d14e664139
</commit_message>
<xml_diff>
--- a/latest/Execution_Summary.xlsx
+++ b/latest/Execution_Summary.xlsx
@@ -1,17 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
-  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30527"/>
+  <workbookPr filterPrivacy="1"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{660982E0-A979-40CF-8179-09DE3AF0BEFD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
-    <sheet sheetId="1" name="Executive Summary" state="visible" r:id="rId4"/>
+    <sheet name="Executive Summary" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
   <si>
     <t>Metric</t>
   </si>
@@ -32,9 +36,6 @@
   </si>
   <si>
     <t>Pass Percentage</t>
-  </si>
-  <si>
-    <t>98.62%</t>
   </si>
   <si>
     <t>Total Duration</t>
@@ -58,19 +59,19 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="2" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-      <sz val="11"/>
-      <name val="Calibri"/>
     </font>
     <font>
       <b/>
-      <color rgb="FFFFFF"/>
       <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
       <name val="Segoe UI"/>
     </font>
   </fonts>
@@ -83,7 +84,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="1E293B"/>
+        <fgColor rgb="FF1E293B"/>
       </patternFill>
     </fill>
   </fills>
@@ -97,16 +98,16 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="CBD5E1"/>
+        <color rgb="FFCBD5E1"/>
       </left>
       <right style="thin">
-        <color rgb="CBD5E1"/>
+        <color rgb="FFCBD5E1"/>
       </right>
       <top style="thin">
-        <color rgb="CBD5E1"/>
+        <color rgb="FFCBD5E1"/>
       </top>
       <bottom style="medium">
-        <color rgb="94A3B8"/>
+        <color rgb="FF94A3B8"/>
       </bottom>
       <diagonal/>
     </border>
@@ -114,11 +115,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -457,15 +459,15 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B9"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="24" customWidth="1"/>
     <col min="2" max="2" width="22" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="28" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" ht="22.35" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -473,7 +475,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>2</v>
       </c>
@@ -481,64 +483,64 @@
         <v>510</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>3</v>
       </c>
       <c r="B3">
-        <v>499</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+        <v>510</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>4</v>
       </c>
       <c r="B4">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>5</v>
       </c>
       <c r="B5">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>6</v>
       </c>
-      <c r="B6" t="s">
+      <c r="B6" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
+      <c r="B7" t="s">
         <v>8</v>
       </c>
-      <c r="B7" t="s">
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
+      <c r="B8" t="s">
         <v>10</v>
       </c>
-      <c r="B8" t="s">
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
+      <c r="B9" t="s">
         <v>12</v>
-      </c>
-      <c r="B9" t="s">
-        <v>13</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
</xml_diff>